<commit_message>
edited WTT.xlsx sections as cut&sew
</commit_message>
<xml_diff>
--- a/data/WTT.xlsx
+++ b/data/WTT.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19070" windowHeight="5740" tabRatio="849" firstSheet="3" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19070" windowHeight="5740" tabRatio="849"/>
   </bookViews>
   <sheets>
     <sheet name="WTT" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11925" uniqueCount="1320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11925" uniqueCount="1321">
   <si>
     <t>Location</t>
   </si>
@@ -4011,6 +4011,9 @@
   </si>
   <si>
     <t>TOTAL STITCHERS REQD.</t>
+  </si>
+  <si>
+    <t>Cut&amp;Sew</t>
   </si>
 </sst>
 </file>
@@ -9909,7 +9912,7 @@
         <v>21</v>
       </c>
       <c r="C98" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D98">
         <v>1</v>
@@ -9971,7 +9974,7 @@
         <v>21</v>
       </c>
       <c r="C99" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D99">
         <v>2</v>
@@ -10033,7 +10036,7 @@
         <v>21</v>
       </c>
       <c r="C100" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D100">
         <v>3</v>
@@ -10095,7 +10098,7 @@
         <v>21</v>
       </c>
       <c r="C101" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D101">
         <v>4</v>
@@ -10157,7 +10160,7 @@
         <v>21</v>
       </c>
       <c r="C102" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D102">
         <v>5</v>
@@ -10219,7 +10222,7 @@
         <v>21</v>
       </c>
       <c r="C103" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D103">
         <v>6</v>
@@ -10281,7 +10284,7 @@
         <v>21</v>
       </c>
       <c r="C104" t="s">
-        <v>199</v>
+        <v>1320</v>
       </c>
       <c r="D104">
         <v>7</v>
@@ -10343,7 +10346,7 @@
         <v>21</v>
       </c>
       <c r="C105" t="s">
-        <v>210</v>
+        <v>1320</v>
       </c>
       <c r="D105">
         <v>8</v>
@@ -10405,7 +10408,7 @@
         <v>21</v>
       </c>
       <c r="C106" t="s">
-        <v>210</v>
+        <v>1320</v>
       </c>
       <c r="D106">
         <v>9</v>
@@ -10467,7 +10470,7 @@
         <v>21</v>
       </c>
       <c r="C107" t="s">
-        <v>210</v>
+        <v>1320</v>
       </c>
       <c r="D107">
         <v>10</v>
@@ -10529,7 +10532,7 @@
         <v>21</v>
       </c>
       <c r="C108" t="s">
-        <v>210</v>
+        <v>1320</v>
       </c>
       <c r="D108">
         <v>11</v>
@@ -10591,7 +10594,7 @@
         <v>21</v>
       </c>
       <c r="C109" t="s">
-        <v>210</v>
+        <v>1320</v>
       </c>
       <c r="D109">
         <v>12</v>
@@ -10653,7 +10656,7 @@
         <v>21</v>
       </c>
       <c r="C110" t="s">
-        <v>218</v>
+        <v>1320</v>
       </c>
       <c r="D110">
         <v>13</v>
@@ -10715,7 +10718,7 @@
         <v>21</v>
       </c>
       <c r="C111" t="s">
-        <v>218</v>
+        <v>1320</v>
       </c>
       <c r="D111">
         <v>14</v>
@@ -10777,7 +10780,7 @@
         <v>21</v>
       </c>
       <c r="C112" t="s">
-        <v>222</v>
+        <v>1320</v>
       </c>
       <c r="D112">
         <v>15</v>
@@ -10839,7 +10842,7 @@
         <v>21</v>
       </c>
       <c r="C113" t="s">
-        <v>222</v>
+        <v>1320</v>
       </c>
       <c r="D113">
         <v>16</v>
@@ -10901,7 +10904,7 @@
         <v>21</v>
       </c>
       <c r="C114" t="s">
-        <v>222</v>
+        <v>1320</v>
       </c>
       <c r="D114">
         <v>17</v>
@@ -10963,7 +10966,7 @@
         <v>21</v>
       </c>
       <c r="C115" t="s">
-        <v>227</v>
+        <v>1320</v>
       </c>
       <c r="D115">
         <v>18</v>
@@ -11025,7 +11028,7 @@
         <v>21</v>
       </c>
       <c r="C116" t="s">
-        <v>227</v>
+        <v>1320</v>
       </c>
       <c r="D116">
         <v>19</v>
@@ -11087,7 +11090,7 @@
         <v>21</v>
       </c>
       <c r="C117" t="s">
-        <v>227</v>
+        <v>1320</v>
       </c>
       <c r="D117">
         <v>20</v>
@@ -11149,7 +11152,7 @@
         <v>21</v>
       </c>
       <c r="C118" t="s">
-        <v>227</v>
+        <v>1320</v>
       </c>
       <c r="D118">
         <v>21</v>
@@ -11211,7 +11214,7 @@
         <v>21</v>
       </c>
       <c r="C119" t="s">
-        <v>236</v>
+        <v>1320</v>
       </c>
       <c r="D119">
         <v>22</v>
@@ -11273,7 +11276,7 @@
         <v>21</v>
       </c>
       <c r="C120" t="s">
-        <v>236</v>
+        <v>1320</v>
       </c>
       <c r="D120">
         <v>23</v>
@@ -11335,7 +11338,7 @@
         <v>21</v>
       </c>
       <c r="C121" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D121">
         <v>24</v>
@@ -11397,7 +11400,7 @@
         <v>21</v>
       </c>
       <c r="C122" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D122">
         <v>25</v>
@@ -11459,7 +11462,7 @@
         <v>21</v>
       </c>
       <c r="C123" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D123">
         <v>26</v>
@@ -11521,7 +11524,7 @@
         <v>21</v>
       </c>
       <c r="C124" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D124">
         <v>27</v>
@@ -11583,7 +11586,7 @@
         <v>21</v>
       </c>
       <c r="C125" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D125">
         <v>28</v>
@@ -11645,7 +11648,7 @@
         <v>21</v>
       </c>
       <c r="C126" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D126">
         <v>29</v>
@@ -11707,7 +11710,7 @@
         <v>21</v>
       </c>
       <c r="C127" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D127">
         <v>30</v>
@@ -11769,7 +11772,7 @@
         <v>21</v>
       </c>
       <c r="C128" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D128">
         <v>31</v>
@@ -11831,7 +11834,7 @@
         <v>21</v>
       </c>
       <c r="C129" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D129">
         <v>32</v>
@@ -11893,7 +11896,7 @@
         <v>21</v>
       </c>
       <c r="C130" t="s">
-        <v>240</v>
+        <v>1320</v>
       </c>
       <c r="D130">
         <v>33</v>
@@ -11955,7 +11958,7 @@
         <v>21</v>
       </c>
       <c r="C131" t="s">
-        <v>252</v>
+        <v>1320</v>
       </c>
       <c r="D131">
         <v>34</v>
@@ -12017,7 +12020,7 @@
         <v>21</v>
       </c>
       <c r="C132" t="s">
-        <v>254</v>
+        <v>1320</v>
       </c>
       <c r="D132">
         <v>35</v>
@@ -12079,7 +12082,7 @@
         <v>21</v>
       </c>
       <c r="C133" t="s">
-        <v>256</v>
+        <v>1320</v>
       </c>
       <c r="D133">
         <v>36</v>
@@ -12141,7 +12144,7 @@
         <v>21</v>
       </c>
       <c r="C134" t="s">
-        <v>256</v>
+        <v>1320</v>
       </c>
       <c r="D134">
         <v>37</v>
@@ -12203,7 +12206,7 @@
         <v>21</v>
       </c>
       <c r="C135" t="s">
-        <v>259</v>
+        <v>1320</v>
       </c>
       <c r="D135">
         <v>38</v>
@@ -12265,7 +12268,7 @@
         <v>21</v>
       </c>
       <c r="C136" t="s">
-        <v>259</v>
+        <v>1320</v>
       </c>
       <c r="D136">
         <v>39</v>
@@ -12327,7 +12330,7 @@
         <v>21</v>
       </c>
       <c r="C137" t="s">
-        <v>259</v>
+        <v>1320</v>
       </c>
       <c r="D137">
         <v>40</v>
@@ -12389,7 +12392,7 @@
         <v>21</v>
       </c>
       <c r="C138" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D138">
         <v>41</v>
@@ -12451,7 +12454,7 @@
         <v>21</v>
       </c>
       <c r="C139" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D139">
         <v>42</v>
@@ -12513,7 +12516,7 @@
         <v>21</v>
       </c>
       <c r="C140" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D140">
         <v>43</v>
@@ -12575,7 +12578,7 @@
         <v>21</v>
       </c>
       <c r="C141" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D141">
         <v>44</v>
@@ -12637,7 +12640,7 @@
         <v>21</v>
       </c>
       <c r="C142" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D142">
         <v>45</v>
@@ -12699,7 +12702,7 @@
         <v>21</v>
       </c>
       <c r="C143" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D143">
         <v>46</v>
@@ -12761,7 +12764,7 @@
         <v>21</v>
       </c>
       <c r="C144" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D144">
         <v>47</v>
@@ -12823,7 +12826,7 @@
         <v>21</v>
       </c>
       <c r="C145" t="s">
-        <v>264</v>
+        <v>1320</v>
       </c>
       <c r="D145">
         <v>48</v>
@@ -12885,7 +12888,7 @@
         <v>21</v>
       </c>
       <c r="C146" t="s">
-        <v>275</v>
+        <v>1320</v>
       </c>
       <c r="D146">
         <v>49</v>
@@ -12947,7 +12950,7 @@
         <v>21</v>
       </c>
       <c r="C147" t="s">
-        <v>278</v>
+        <v>1320</v>
       </c>
       <c r="D147">
         <v>50</v>
@@ -13009,7 +13012,7 @@
         <v>21</v>
       </c>
       <c r="C148" t="s">
-        <v>281</v>
+        <v>1320</v>
       </c>
       <c r="D148">
         <v>51</v>
@@ -18755,7 +18758,7 @@
         <v>3</v>
       </c>
       <c r="F6">
-        <f>SUM(B6:E6)</f>
+        <f t="shared" ref="F6:F11" si="0">SUM(B6:E6)</f>
         <v>93</v>
       </c>
     </row>
@@ -18776,7 +18779,7 @@
         <v>5</v>
       </c>
       <c r="F7">
-        <f>SUM(B7:E7)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
@@ -18801,7 +18804,7 @@
         <v>1</v>
       </c>
       <c r="F8">
-        <f>SUM(B8:E8)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
@@ -18818,15 +18821,15 @@
         <v>9</v>
       </c>
       <c r="D9" s="3">
-        <f t="shared" ref="D9:E9" si="0">D8*3</f>
+        <f t="shared" ref="D9:E9" si="1">D8*3</f>
         <v>6</v>
       </c>
       <c r="E9" s="3">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="F9" s="3">
-        <f>SUM(B9:E9)</f>
         <v>24</v>
       </c>
     </row>
@@ -18839,19 +18842,19 @@
         <v>9</v>
       </c>
       <c r="C10">
-        <f t="shared" ref="C10:E10" si="1">ROUNDUP(C2/24,0)*3</f>
+        <f t="shared" ref="C10:E10" si="2">ROUNDUP(C2/24,0)*3</f>
         <v>12</v>
       </c>
       <c r="D10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="E10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="F10">
-        <f>SUM(B10:E10)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
@@ -18864,7 +18867,7 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:E11" si="2">ROUNDUP(C2/28,0)*3</f>
+        <f t="shared" ref="C11:E11" si="3">ROUNDUP(C2/28,0)*3</f>
         <v>12</v>
       </c>
       <c r="D11">
@@ -18872,11 +18875,11 @@
         <v>6</v>
       </c>
       <c r="E11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="F11">
-        <f>SUM(B11:E11)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>

</xml_diff>